<commit_message>
Commit At 2026-09-23 20:34:11
</commit_message>
<xml_diff>
--- a/数据/无人机应急物资运输基础数据/中继无人机数据.xlsx
+++ b/数据/无人机应急物资运输基础数据/中继无人机数据.xlsx
@@ -5,16 +5,14 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SF_Dir\第二十三届中国研究生数学建模竞赛 - 中文题目\中文题目\D题\数据\无人机应急物资运输基础数据\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HH\Desktop\(南航学习资料汇总)博四下结束暑假\赛题+参考答案 - 最终版本\赛题+参考答案 - 最终版本\赛题\数据\无人机应急物资运输基础数据\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="25600" windowHeight="12080"/>
+    <workbookView windowWidth="30720" windowHeight="13380"/>
   </bookViews>
   <sheets>
-    <sheet name="中继机型参数 " sheetId="1" r:id="rId1"/>
-    <sheet name="逐架中继无人机清单 " sheetId="2" r:id="rId2"/>
-    <sheet name="共享能源组件库存 " sheetId="3" r:id="rId3"/>
+    <sheet name="数据" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +32,19 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="31">
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>中继机型参数</t>
+    </r>
+  </si>
   <si>
     <r>
       <rPr>
@@ -528,6 +538,18 @@
   <si>
     <r>
       <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>逐架中继无人机清单</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="宋体"/>
@@ -555,6 +577,18 @@
   </si>
   <si>
     <t>R02</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
+      <t>共享能源组件库存</t>
+    </r>
   </si>
   <si>
     <r>
@@ -608,13 +642,19 @@
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="0.0"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="28">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
       <charset val="134"/>
     </font>
     <font>
+      <sz val="11"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
@@ -622,12 +662,13 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
       <name val="Times New Roman"/>
       <charset val="134"/>
     </font>
@@ -783,6 +824,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="宋体"/>
@@ -1099,199 +1147,199 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="49" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="49" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="50">
@@ -1764,343 +1812,321 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:S11"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
+  <dimension ref="A1:S12"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="24.1" style="6" customWidth="1"/>
-    <col min="2" max="2" width="24" style="6" customWidth="1"/>
-    <col min="3" max="3" width="25.1" style="6" customWidth="1"/>
-    <col min="4" max="4" width="22.5" style="6" customWidth="1"/>
-    <col min="5" max="5" width="20.8" style="6" customWidth="1"/>
-    <col min="6" max="6" width="19" style="6" customWidth="1"/>
-    <col min="7" max="7" width="16" style="6" customWidth="1"/>
-    <col min="8" max="8" width="24.4" style="6" customWidth="1"/>
-    <col min="9" max="9" width="18.4" style="6" customWidth="1"/>
-    <col min="10" max="10" width="20.4" style="6" customWidth="1"/>
-    <col min="11" max="11" width="14" style="6" customWidth="1"/>
-    <col min="12" max="12" width="16" style="6" customWidth="1"/>
-    <col min="13" max="13" width="18.8" style="6" customWidth="1"/>
-    <col min="14" max="14" width="18.6" style="6" customWidth="1"/>
-    <col min="15" max="16" width="14" style="6" customWidth="1"/>
-    <col min="17" max="17" width="17.6" style="6" customWidth="1"/>
-    <col min="18" max="18" width="20" style="6" customWidth="1"/>
-    <col min="19" max="19" width="22" style="6" customWidth="1"/>
-    <col min="20" max="16384" width="9" style="6"/>
+    <col min="1" max="1" width="24.1" style="1" customWidth="1"/>
+    <col min="2" max="2" width="24" style="1" customWidth="1"/>
+    <col min="3" max="3" width="25.1" style="1" customWidth="1"/>
+    <col min="4" max="4" width="22.5" style="1" customWidth="1"/>
+    <col min="5" max="5" width="20.8" style="1" customWidth="1"/>
+    <col min="6" max="6" width="19" style="1" customWidth="1"/>
+    <col min="7" max="7" width="16" style="1" customWidth="1"/>
+    <col min="8" max="8" width="24.4" style="1" customWidth="1"/>
+    <col min="9" max="9" width="18.4" style="1" customWidth="1"/>
+    <col min="10" max="10" width="20.4" style="1" customWidth="1"/>
+    <col min="11" max="11" width="14" style="1" customWidth="1"/>
+    <col min="12" max="12" width="16" style="1" customWidth="1"/>
+    <col min="13" max="13" width="18.8" style="1" customWidth="1"/>
+    <col min="14" max="14" width="18.6" style="1" customWidth="1"/>
+    <col min="15" max="16" width="14" style="1" customWidth="1"/>
+    <col min="17" max="17" width="17.6" style="1" customWidth="1"/>
+    <col min="18" max="18" width="20" style="1" customWidth="1"/>
+    <col min="19" max="19" width="22" style="1" customWidth="1"/>
+    <col min="20" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1" spans="1:19">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="24" customHeight="1" spans="1:19">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+      <c r="S1" s="2"/>
+    </row>
+    <row r="2" ht="32" customHeight="1" spans="1:19">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="C2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="D2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="E2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="F2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="G2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="H2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="I2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="J2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="K2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="L2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="M2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="N2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="O2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="P2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="Q2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="7" t="s">
+      <c r="R2" s="3" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="2" ht="22" customHeight="1" spans="1:19">
-      <c r="A2" s="2" t="s">
+      <c r="S2" s="4" t="s">
         <v>19</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C2" s="8">
-        <v>21</v>
-      </c>
-      <c r="D2" s="8">
-        <v>2.5</v>
-      </c>
-      <c r="E2" s="8">
-        <v>23.5</v>
-      </c>
-      <c r="F2" s="8">
-        <v>15</v>
-      </c>
-      <c r="G2" s="9">
-        <v>1.15</v>
-      </c>
-      <c r="H2" s="9">
-        <v>3.2</v>
-      </c>
-      <c r="I2" s="3">
-        <v>20</v>
-      </c>
-      <c r="J2" s="3">
-        <v>180</v>
-      </c>
-      <c r="K2" s="3">
-        <v>30</v>
-      </c>
-      <c r="L2" s="3">
-        <v>300</v>
-      </c>
-      <c r="M2" s="3">
-        <v>4</v>
-      </c>
-      <c r="N2" s="3">
-        <v>3</v>
-      </c>
-      <c r="O2" s="9">
-        <v>0.72</v>
-      </c>
-      <c r="P2" s="9">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="9">
-        <v>1.05</v>
-      </c>
-      <c r="R2" s="9">
-        <v>0.05</v>
-      </c>
-      <c r="S2" s="10">
-        <v>300</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:19">
-      <c r="A3" s="11"/>
-      <c r="B3" s="11"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
-      <c r="O3" s="13"/>
-      <c r="P3" s="13"/>
-      <c r="Q3" s="13"/>
-      <c r="R3" s="13"/>
-      <c r="S3" s="15"/>
+      <c r="A3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" s="6">
+        <v>21</v>
+      </c>
+      <c r="D3" s="6">
+        <v>2.5</v>
+      </c>
+      <c r="E3" s="6">
+        <v>23.5</v>
+      </c>
+      <c r="F3" s="6">
+        <v>15</v>
+      </c>
+      <c r="G3" s="7">
+        <v>1.15</v>
+      </c>
+      <c r="H3" s="7">
+        <v>3.2</v>
+      </c>
+      <c r="I3" s="8">
+        <v>20</v>
+      </c>
+      <c r="J3" s="8">
+        <v>180</v>
+      </c>
+      <c r="K3" s="8">
+        <v>30</v>
+      </c>
+      <c r="L3" s="8">
+        <v>300</v>
+      </c>
+      <c r="M3" s="8">
+        <v>4</v>
+      </c>
+      <c r="N3" s="8">
+        <v>3</v>
+      </c>
+      <c r="O3" s="7">
+        <v>0.72</v>
+      </c>
+      <c r="P3" s="7">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="7">
+        <v>1.05</v>
+      </c>
+      <c r="R3" s="7">
+        <v>0.05</v>
+      </c>
+      <c r="S3" s="9">
+        <v>300</v>
+      </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:19">
-      <c r="A4" s="16"/>
-      <c r="B4" s="16"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="12"/>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="14"/>
-      <c r="J4" s="14"/>
-      <c r="K4" s="14"/>
-      <c r="L4" s="14"/>
-      <c r="M4" s="14"/>
-      <c r="N4" s="14"/>
-      <c r="O4" s="13"/>
-      <c r="P4" s="13"/>
-      <c r="Q4" s="13"/>
-      <c r="R4" s="13"/>
-      <c r="S4" s="15"/>
+      <c r="A4" s="10"/>
+      <c r="B4" s="10"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="13"/>
+      <c r="J4" s="13"/>
+      <c r="K4" s="13"/>
+      <c r="L4" s="13"/>
+      <c r="M4" s="13"/>
+      <c r="N4" s="13"/>
+      <c r="O4" s="12"/>
+      <c r="P4" s="12"/>
+      <c r="Q4" s="12"/>
+      <c r="R4" s="12"/>
+      <c r="S4" s="14"/>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:19">
-      <c r="A5" s="16"/>
-      <c r="B5" s="16"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="13"/>
-      <c r="H5" s="13"/>
-      <c r="I5" s="14"/>
-      <c r="J5" s="14"/>
-      <c r="K5" s="14"/>
-      <c r="L5" s="14"/>
-      <c r="M5" s="14"/>
-      <c r="N5" s="14"/>
-      <c r="O5" s="13"/>
-      <c r="P5" s="13"/>
-      <c r="Q5" s="13"/>
-      <c r="R5" s="13"/>
-      <c r="S5" s="15"/>
+      <c r="A5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="12"/>
+      <c r="I5" s="13"/>
+      <c r="J5" s="13"/>
+      <c r="K5" s="13"/>
+      <c r="L5" s="13"/>
+      <c r="M5" s="13"/>
+      <c r="N5" s="13"/>
+      <c r="O5" s="12"/>
+      <c r="P5" s="12"/>
+      <c r="Q5" s="12"/>
+      <c r="R5" s="12"/>
+      <c r="S5" s="14"/>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:19">
-      <c r="A6" s="16"/>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="13"/>
-      <c r="H6" s="13"/>
-      <c r="I6" s="14"/>
-      <c r="J6" s="14"/>
-      <c r="K6" s="14"/>
-      <c r="L6" s="14"/>
-      <c r="M6" s="14"/>
-      <c r="N6" s="14"/>
-      <c r="O6" s="13"/>
-      <c r="P6" s="13"/>
-      <c r="Q6" s="13"/>
-      <c r="R6" s="13"/>
-      <c r="S6" s="15"/>
+      <c r="A6" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" s="11"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="12"/>
+      <c r="H6" s="12"/>
+      <c r="I6" s="13"/>
+      <c r="J6" s="13"/>
+      <c r="K6" s="13"/>
+      <c r="L6" s="13"/>
+      <c r="M6" s="13"/>
+      <c r="N6" s="13"/>
+      <c r="O6" s="12"/>
+      <c r="P6" s="12"/>
+      <c r="Q6" s="12"/>
+      <c r="R6" s="12"/>
+      <c r="S6" s="14"/>
     </row>
-    <row r="7" spans="1:19">
-      <c r="A7" s="16"/>
-      <c r="B7" s="16"/>
-      <c r="C7" s="16"/>
+    <row r="7" ht="22" customHeight="1" spans="1:19">
+      <c r="A7" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="12"/>
+      <c r="I7" s="13"/>
+      <c r="J7" s="13"/>
+      <c r="K7" s="13"/>
+      <c r="L7" s="13"/>
+      <c r="M7" s="13"/>
+      <c r="N7" s="13"/>
+      <c r="O7" s="12"/>
+      <c r="P7" s="12"/>
+      <c r="Q7" s="12"/>
+      <c r="R7" s="12"/>
+      <c r="S7" s="14"/>
     </row>
     <row r="8" spans="1:19">
-      <c r="A8" s="16"/>
-      <c r="B8" s="16"/>
-      <c r="C8" s="16"/>
+      <c r="A8" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="9" ht="24" customHeight="1" spans="1:19">
-      <c r="A9" s="16"/>
-      <c r="B9" s="16"/>
-      <c r="C9" s="16"/>
+    <row r="9" spans="1:19">
+      <c r="A9" s="5"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
     </row>
-    <row r="10" ht="32" customHeight="1" spans="1:19">
-      <c r="A10" s="16"/>
-      <c r="B10" s="16"/>
-      <c r="C10" s="16"/>
+    <row r="10" ht="24" customHeight="1" spans="1:19">
+      <c r="A10" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
     </row>
-    <row r="11" ht="22" customHeight="1" spans="1:19">
-      <c r="A11" s="16"/>
-      <c r="B11" s="16"/>
-      <c r="C11" s="16"/>
+    <row r="11" ht="32" customHeight="1" spans="1:19">
+      <c r="A11" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1" spans="1:19">
+      <c r="A12" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="8">
+        <v>6</v>
+      </c>
+      <c r="C12" s="16">
+        <v>1800</v>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:S1"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A10:C10"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.66666666666667" defaultRowHeight="14" outlineLevelRow="3" outlineLevelCol="2"/>
-  <sheetData>
-    <row r="1" ht="28" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.66666666666667" defaultRowHeight="14" outlineLevelRow="1" outlineLevelCol="2"/>
-  <sheetData>
-    <row r="1" ht="42" spans="1:3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B2" s="3">
-        <v>6</v>
-      </c>
-      <c r="C2" s="4">
-        <v>1800</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
-</worksheet>
 </file>
</xml_diff>